<commit_message>
darkmode and ui tweaks
</commit_message>
<xml_diff>
--- a/public/DocumentTrackingLog.xlsx
+++ b/public/DocumentTrackingLog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shelt\Projects\CheckMate-Vite\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3F51E2B-7DB6-4A42-946D-56AE836FF8B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5823B987-E205-4901-9F97-910CC2037E2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracking Log" sheetId="1" r:id="rId1"/>
@@ -771,8 +771,19 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -813,6 +824,26 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="10" borderId="2" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="10" borderId="3" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -824,32 +855,12 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="10" borderId="2" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="10" borderId="3" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -865,19 +876,8 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1537,43 +1537,58 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultColWidth="19.88671875" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.109375" style="12" customWidth="1"/>
-    <col min="2" max="2" width="22.6640625" style="12" customWidth="1"/>
-    <col min="3" max="3" width="32.44140625" style="12" customWidth="1"/>
-    <col min="4" max="4" width="34.33203125" style="12" customWidth="1"/>
-    <col min="5" max="5" width="33.109375" style="12" customWidth="1"/>
-    <col min="6" max="6" width="24.44140625" style="12" customWidth="1"/>
-    <col min="7" max="7" width="41.33203125" style="12" customWidth="1"/>
-    <col min="8" max="8" width="18.44140625" style="12" customWidth="1"/>
-    <col min="9" max="9" width="16.6640625" style="12" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" style="78" customWidth="1"/>
+    <col min="3" max="3" width="32.44140625" style="78" customWidth="1"/>
+    <col min="4" max="4" width="34.33203125" style="78" customWidth="1"/>
+    <col min="5" max="5" width="33.109375" style="78" customWidth="1"/>
+    <col min="6" max="6" width="24.44140625" style="78" customWidth="1"/>
+    <col min="7" max="7" width="41.33203125" style="78" customWidth="1"/>
+    <col min="8" max="8" width="18.44140625" style="78" customWidth="1"/>
+    <col min="9" max="9" width="16.6640625" style="78" customWidth="1"/>
     <col min="10" max="10" width="2.33203125" style="12" hidden="1" customWidth="1"/>
     <col min="11" max="16383" width="19.88671875" style="12" customWidth="1"/>
     <col min="16384" max="16384" width="19.88671875" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
       <c r="G1" s="13"/>
-      <c r="H1" s="53" t="s">
+      <c r="H1" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="53"/>
+      <c r="I1" s="56"/>
     </row>
     <row r="2" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
       <c r="G2" s="13"/>
-      <c r="H2" s="54" t="s">
+      <c r="H2" s="57" t="s">
         <v>55</v>
       </c>
-      <c r="I2" s="54"/>
+      <c r="I2" s="57"/>
     </row>
     <row r="3" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
       <c r="G3" s="13"/>
-      <c r="H3" s="54" t="s">
+      <c r="H3" s="57" t="s">
         <v>56</v>
       </c>
-      <c r="I3" s="54"/>
+      <c r="I3" s="57"/>
     </row>
     <row r="4" spans="1:9" s="3" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="12"/>
@@ -1583,23 +1598,23 @@
       <c r="E4" s="12"/>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
-      <c r="H4" s="54" t="s">
+      <c r="H4" s="57" t="s">
         <v>57</v>
       </c>
-      <c r="I4" s="54"/>
+      <c r="I4" s="57"/>
     </row>
     <row r="5" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="14"/>
-      <c r="B5" s="55" t="s">
+      <c r="B5" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="55"/>
-      <c r="D5" s="55"/>
-      <c r="E5" s="55"/>
-      <c r="F5" s="55"/>
-      <c r="G5" s="55"/>
-      <c r="H5" s="55"/>
-      <c r="I5" s="55"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="58"/>
+      <c r="F5" s="58"/>
+      <c r="G5" s="58"/>
+      <c r="H5" s="58"/>
+      <c r="I5" s="58"/>
     </row>
     <row r="6" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14"/>
@@ -1614,18 +1629,18 @@
     </row>
     <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="14"/>
-      <c r="B7" s="49" t="s">
+      <c r="B7" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="50"/>
+      <c r="C7" s="53"/>
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
       <c r="G7" s="14"/>
-      <c r="H7" s="51" t="s">
+      <c r="H7" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="I7" s="51"/>
+      <c r="I7" s="54"/>
     </row>
     <row r="8" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14"/>
@@ -1717,10 +1732,10 @@
       <c r="E14" s="14"/>
       <c r="F14" s="14"/>
       <c r="G14" s="14"/>
-      <c r="H14" s="52" t="s">
+      <c r="H14" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="I14" s="52"/>
+      <c r="I14" s="55"/>
     </row>
     <row r="15" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="21" t="s">
@@ -1747,356 +1762,6 @@
       <c r="I15" s="24" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="48"/>
-      <c r="C16" s="48"/>
-      <c r="D16" s="48"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="48"/>
-      <c r="G16" s="48"/>
-      <c r="H16" s="48"/>
-      <c r="I16" s="48"/>
-    </row>
-    <row r="17" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="48"/>
-      <c r="C17" s="48"/>
-      <c r="D17" s="48"/>
-      <c r="E17" s="48"/>
-      <c r="F17" s="48"/>
-      <c r="G17" s="48"/>
-      <c r="H17" s="48"/>
-      <c r="I17" s="48"/>
-    </row>
-    <row r="18" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="48"/>
-      <c r="C18" s="48"/>
-      <c r="D18" s="48"/>
-      <c r="E18" s="48"/>
-      <c r="F18" s="48"/>
-      <c r="G18" s="48"/>
-      <c r="H18" s="48"/>
-      <c r="I18" s="48"/>
-    </row>
-    <row r="19" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="48"/>
-      <c r="C19" s="48"/>
-      <c r="D19" s="48"/>
-      <c r="E19" s="48"/>
-      <c r="F19" s="48"/>
-      <c r="G19" s="48"/>
-      <c r="H19" s="48"/>
-      <c r="I19" s="48"/>
-    </row>
-    <row r="20" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="48"/>
-      <c r="C20" s="48"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="48"/>
-      <c r="H20" s="48"/>
-      <c r="I20" s="48"/>
-    </row>
-    <row r="21" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="48"/>
-      <c r="C21" s="48"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="48"/>
-      <c r="G21" s="48"/>
-      <c r="H21" s="48"/>
-      <c r="I21" s="48"/>
-    </row>
-    <row r="22" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="48"/>
-      <c r="C22" s="48"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="48"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="48"/>
-      <c r="H22" s="48"/>
-      <c r="I22" s="48"/>
-    </row>
-    <row r="23" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="48"/>
-      <c r="C23" s="48"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="48"/>
-      <c r="G23" s="48"/>
-      <c r="H23" s="48"/>
-      <c r="I23" s="48"/>
-    </row>
-    <row r="24" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="48"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="48"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="48"/>
-    </row>
-    <row r="25" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="48"/>
-      <c r="C25" s="48"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="48"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="48"/>
-      <c r="H25" s="48"/>
-      <c r="I25" s="48"/>
-    </row>
-    <row r="26" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="48"/>
-      <c r="C26" s="48"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="48"/>
-      <c r="G26" s="48"/>
-      <c r="H26" s="48"/>
-      <c r="I26" s="48"/>
-    </row>
-    <row r="27" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="48"/>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="48"/>
-      <c r="I27" s="48"/>
-    </row>
-    <row r="28" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="48"/>
-      <c r="C28" s="48"/>
-      <c r="D28" s="48"/>
-      <c r="E28" s="48"/>
-      <c r="F28" s="48"/>
-      <c r="G28" s="48"/>
-      <c r="H28" s="48"/>
-      <c r="I28" s="48"/>
-    </row>
-    <row r="29" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="48"/>
-      <c r="C29" s="48"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="48"/>
-      <c r="F29" s="48"/>
-      <c r="G29" s="48"/>
-      <c r="H29" s="48"/>
-      <c r="I29" s="48"/>
-    </row>
-    <row r="30" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="48"/>
-      <c r="C30" s="48"/>
-      <c r="D30" s="48"/>
-      <c r="E30" s="48"/>
-      <c r="F30" s="48"/>
-      <c r="G30" s="48"/>
-      <c r="H30" s="48"/>
-      <c r="I30" s="48"/>
-    </row>
-    <row r="31" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="48"/>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="48"/>
-      <c r="G31" s="48"/>
-      <c r="H31" s="48"/>
-      <c r="I31" s="48"/>
-    </row>
-    <row r="32" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="48"/>
-      <c r="C32" s="48"/>
-      <c r="D32" s="48"/>
-      <c r="E32" s="48"/>
-      <c r="F32" s="48"/>
-      <c r="G32" s="48"/>
-      <c r="H32" s="48"/>
-      <c r="I32" s="48"/>
-    </row>
-    <row r="33" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="48"/>
-      <c r="C33" s="48"/>
-      <c r="D33" s="48"/>
-      <c r="E33" s="48"/>
-      <c r="F33" s="48"/>
-      <c r="G33" s="48"/>
-      <c r="H33" s="48"/>
-      <c r="I33" s="48"/>
-    </row>
-    <row r="34" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="48"/>
-      <c r="C34" s="48"/>
-      <c r="D34" s="48"/>
-      <c r="E34" s="48"/>
-      <c r="F34" s="48"/>
-      <c r="G34" s="48"/>
-      <c r="H34" s="48"/>
-      <c r="I34" s="48"/>
-    </row>
-    <row r="35" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="48"/>
-      <c r="C35" s="48"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="48"/>
-      <c r="F35" s="48"/>
-      <c r="G35" s="48"/>
-      <c r="H35" s="48"/>
-      <c r="I35" s="48"/>
-    </row>
-    <row r="36" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="48"/>
-      <c r="C36" s="48"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="48"/>
-      <c r="F36" s="48"/>
-      <c r="G36" s="48"/>
-      <c r="H36" s="48"/>
-      <c r="I36" s="48"/>
-    </row>
-    <row r="37" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="48"/>
-      <c r="C37" s="48"/>
-      <c r="D37" s="48"/>
-      <c r="E37" s="48"/>
-      <c r="F37" s="48"/>
-      <c r="G37" s="48"/>
-      <c r="H37" s="48"/>
-      <c r="I37" s="48"/>
-    </row>
-    <row r="38" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="48"/>
-      <c r="C38" s="48"/>
-      <c r="D38" s="48"/>
-      <c r="E38" s="48"/>
-      <c r="F38" s="48"/>
-      <c r="G38" s="48"/>
-      <c r="H38" s="48"/>
-      <c r="I38" s="48"/>
-    </row>
-    <row r="39" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="48"/>
-      <c r="C39" s="48"/>
-      <c r="D39" s="48"/>
-      <c r="E39" s="48"/>
-      <c r="F39" s="48"/>
-      <c r="G39" s="48"/>
-      <c r="H39" s="48"/>
-      <c r="I39" s="48"/>
-    </row>
-    <row r="40" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="48"/>
-      <c r="C40" s="48"/>
-      <c r="D40" s="48"/>
-      <c r="E40" s="48"/>
-      <c r="F40" s="48"/>
-      <c r="G40" s="48"/>
-      <c r="H40" s="48"/>
-      <c r="I40" s="48"/>
-    </row>
-    <row r="41" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="48"/>
-      <c r="C41" s="48"/>
-      <c r="D41" s="48"/>
-      <c r="E41" s="48"/>
-      <c r="F41" s="48"/>
-      <c r="G41" s="48"/>
-      <c r="H41" s="48"/>
-      <c r="I41" s="48"/>
-    </row>
-    <row r="42" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="48"/>
-      <c r="C42" s="48"/>
-      <c r="D42" s="48"/>
-      <c r="E42" s="48"/>
-      <c r="F42" s="48"/>
-      <c r="G42" s="48"/>
-      <c r="H42" s="48"/>
-      <c r="I42" s="48"/>
-    </row>
-    <row r="43" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="48"/>
-      <c r="C43" s="48"/>
-      <c r="D43" s="48"/>
-      <c r="E43" s="48"/>
-      <c r="F43" s="48"/>
-      <c r="G43" s="48"/>
-      <c r="H43" s="48"/>
-      <c r="I43" s="48"/>
-    </row>
-    <row r="44" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="48"/>
-      <c r="C44" s="48"/>
-      <c r="D44" s="48"/>
-      <c r="E44" s="48"/>
-      <c r="F44" s="48"/>
-      <c r="G44" s="48"/>
-      <c r="H44" s="48"/>
-      <c r="I44" s="48"/>
-    </row>
-    <row r="45" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="48"/>
-      <c r="C45" s="48"/>
-      <c r="D45" s="48"/>
-      <c r="E45" s="48"/>
-      <c r="F45" s="48"/>
-      <c r="G45" s="48"/>
-      <c r="H45" s="48"/>
-      <c r="I45" s="48"/>
-    </row>
-    <row r="46" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="48"/>
-      <c r="C46" s="48"/>
-      <c r="D46" s="48"/>
-      <c r="E46" s="48"/>
-      <c r="F46" s="48"/>
-      <c r="G46" s="48"/>
-      <c r="H46" s="48"/>
-      <c r="I46" s="48"/>
-    </row>
-    <row r="47" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="48"/>
-      <c r="C47" s="48"/>
-      <c r="D47" s="48"/>
-      <c r="E47" s="48"/>
-      <c r="F47" s="48"/>
-      <c r="G47" s="48"/>
-      <c r="H47" s="48"/>
-      <c r="I47" s="48"/>
-    </row>
-    <row r="48" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="48"/>
-      <c r="C48" s="48"/>
-      <c r="D48" s="48"/>
-      <c r="E48" s="48"/>
-      <c r="F48" s="48"/>
-      <c r="G48" s="48"/>
-      <c r="H48" s="48"/>
-      <c r="I48" s="48"/>
-    </row>
-    <row r="49" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="48"/>
-      <c r="C49" s="48"/>
-      <c r="D49" s="48"/>
-      <c r="E49" s="48"/>
-      <c r="F49" s="48"/>
-      <c r="G49" s="48"/>
-      <c r="H49" s="48"/>
-      <c r="I49" s="48"/>
-    </row>
-    <row r="50" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="48"/>
-      <c r="C50" s="48"/>
-      <c r="D50" s="48"/>
-      <c r="E50" s="48"/>
-      <c r="F50" s="48"/>
-      <c r="G50" s="48"/>
-      <c r="H50" s="48"/>
-      <c r="I50" s="48"/>
     </row>
   </sheetData>
   <sheetProtection insertRows="0" sort="0" autoFilter="0"/>
@@ -2132,47 +1797,75 @@
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" style="25" customWidth="1"/>
-    <col min="2" max="2" width="21" style="25" customWidth="1"/>
-    <col min="3" max="4" width="29.6640625" style="25" customWidth="1"/>
-    <col min="5" max="5" width="21.109375" style="25" customWidth="1"/>
-    <col min="6" max="6" width="24.6640625" style="25" customWidth="1"/>
-    <col min="7" max="7" width="27.5546875" style="25" customWidth="1"/>
-    <col min="8" max="8" width="32.33203125" style="25" customWidth="1"/>
-    <col min="9" max="9" width="35.109375" style="25" customWidth="1"/>
+    <col min="2" max="2" width="21" style="13" customWidth="1"/>
+    <col min="3" max="4" width="29.6640625" style="13" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" style="13" customWidth="1"/>
+    <col min="6" max="6" width="24.6640625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="27.5546875" style="13" customWidth="1"/>
+    <col min="8" max="8" width="32.33203125" style="13" customWidth="1"/>
+    <col min="9" max="9" width="35.109375" style="13" customWidth="1"/>
     <col min="10" max="16384" width="8.88671875" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
       <c r="I1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="2" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
       <c r="I2" s="13" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="3" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
       <c r="I3" s="13" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="4" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
       <c r="I4" s="13" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="5" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="57" t="s">
+      <c r="B5" s="60" t="s">
         <v>58</v>
       </c>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="60"/>
     </row>
     <row r="6" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="26"/>
@@ -2184,21 +1877,39 @@
       <c r="H6" s="26"/>
       <c r="I6" s="26"/>
     </row>
+    <row r="7" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="25"/>
+    </row>
     <row r="8" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="56" t="s">
+      <c r="B8" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="56"/>
-      <c r="H8" s="58" t="s">
+      <c r="C8" s="59"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="I8" s="59"/>
+      <c r="I8" s="62"/>
     </row>
     <row r="9" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="27" t="s">
         <v>2</v>
       </c>
       <c r="C9" s="28"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
       <c r="H9" s="27" t="s">
         <v>20</v>
       </c>
@@ -2209,6 +1920,10 @@
         <v>3</v>
       </c>
       <c r="C10" s="28"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
       <c r="H10" s="27" t="s">
         <v>3</v>
       </c>
@@ -2219,6 +1934,10 @@
         <v>4</v>
       </c>
       <c r="C11" s="28"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
       <c r="H11" s="27" t="s">
         <v>5</v>
       </c>
@@ -2229,6 +1948,10 @@
         <v>6</v>
       </c>
       <c r="C12" s="30"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
       <c r="H12" s="27" t="s">
         <v>21</v>
       </c>
@@ -2239,393 +1962,426 @@
         <v>5</v>
       </c>
       <c r="C13" s="32"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="25"/>
+      <c r="H13" s="25"/>
+      <c r="I13" s="25"/>
     </row>
     <row r="14" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="27" t="s">
         <v>22</v>
       </c>
       <c r="C14" s="33"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="25"/>
+    </row>
+    <row r="15" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
     </row>
     <row r="16" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="34" t="s">
         <v>61</v>
       </c>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
     </row>
     <row r="17" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="25" t="s">
         <v>23</v>
       </c>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
     </row>
     <row r="18" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="25" t="s">
         <v>24</v>
       </c>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
     </row>
     <row r="19" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="75" t="s">
+      <c r="B19" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="75" t="s">
+      <c r="C19" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="75" t="s">
+      <c r="D19" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="E19" s="75" t="s">
+      <c r="E19" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="F19" s="75" t="s">
+      <c r="F19" s="48" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="75" t="s">
+      <c r="G19" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="H19" s="75" t="s">
+      <c r="H19" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="I19" s="75" t="s">
+      <c r="I19" s="48" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="36"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="36"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="36"/>
-      <c r="I20" s="36"/>
     </row>
     <row r="21" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21"/>
-      <c r="B21"/>
-      <c r="C21"/>
-      <c r="D21"/>
-      <c r="E21"/>
-      <c r="F21"/>
-      <c r="G21"/>
-      <c r="H21"/>
-      <c r="I21"/>
+      <c r="B21" s="78"/>
+      <c r="C21" s="78"/>
+      <c r="D21" s="78"/>
+      <c r="E21" s="78"/>
+      <c r="F21" s="78"/>
+      <c r="G21" s="78"/>
+      <c r="H21" s="78"/>
+      <c r="I21" s="78"/>
     </row>
     <row r="22" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22"/>
-      <c r="B22"/>
-      <c r="C22"/>
-      <c r="D22"/>
-      <c r="E22"/>
-      <c r="F22"/>
-      <c r="G22"/>
-      <c r="H22"/>
-      <c r="I22"/>
+      <c r="B22" s="78"/>
+      <c r="C22" s="78"/>
+      <c r="D22" s="78"/>
+      <c r="E22" s="78"/>
+      <c r="F22" s="78"/>
+      <c r="G22" s="78"/>
+      <c r="H22" s="78"/>
+      <c r="I22" s="78"/>
     </row>
     <row r="23" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23"/>
-      <c r="B23"/>
-      <c r="C23"/>
-      <c r="D23"/>
-      <c r="E23"/>
-      <c r="F23"/>
-      <c r="G23"/>
-      <c r="H23"/>
-      <c r="I23"/>
+      <c r="B23" s="78"/>
+      <c r="C23" s="78"/>
+      <c r="D23" s="78"/>
+      <c r="E23" s="78"/>
+      <c r="F23" s="78"/>
+      <c r="G23" s="78"/>
+      <c r="H23" s="78"/>
+      <c r="I23" s="78"/>
     </row>
     <row r="24" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24"/>
-      <c r="B24"/>
-      <c r="C24"/>
-      <c r="D24"/>
-      <c r="E24"/>
-      <c r="F24"/>
-      <c r="G24"/>
-      <c r="H24"/>
-      <c r="I24"/>
+      <c r="B24" s="78"/>
+      <c r="C24" s="78"/>
+      <c r="D24" s="78"/>
+      <c r="E24" s="78"/>
+      <c r="F24" s="78"/>
+      <c r="G24" s="78"/>
+      <c r="H24" s="78"/>
+      <c r="I24" s="78"/>
     </row>
     <row r="25" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25"/>
-      <c r="B25"/>
-      <c r="C25"/>
-      <c r="D25"/>
-      <c r="E25"/>
-      <c r="F25"/>
-      <c r="G25"/>
-      <c r="H25"/>
-      <c r="I25"/>
+      <c r="B25" s="78"/>
+      <c r="C25" s="78"/>
+      <c r="D25" s="78"/>
+      <c r="E25" s="78"/>
+      <c r="F25" s="78"/>
+      <c r="G25" s="78"/>
+      <c r="H25" s="78"/>
+      <c r="I25" s="78"/>
     </row>
     <row r="26" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26"/>
-      <c r="B26"/>
-      <c r="C26"/>
-      <c r="D26"/>
-      <c r="E26"/>
-      <c r="F26"/>
-      <c r="G26"/>
-      <c r="H26"/>
-      <c r="I26"/>
+      <c r="B26" s="78"/>
+      <c r="C26" s="78"/>
+      <c r="D26" s="78"/>
+      <c r="E26" s="78"/>
+      <c r="F26" s="78"/>
+      <c r="G26" s="78"/>
+      <c r="H26" s="78"/>
+      <c r="I26" s="78"/>
     </row>
     <row r="27" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27"/>
-      <c r="B27"/>
-      <c r="C27"/>
-      <c r="D27"/>
-      <c r="E27"/>
-      <c r="F27"/>
-      <c r="G27"/>
-      <c r="H27"/>
-      <c r="I27"/>
+      <c r="B27" s="78"/>
+      <c r="C27" s="78"/>
+      <c r="D27" s="78"/>
+      <c r="E27" s="78"/>
+      <c r="F27" s="78"/>
+      <c r="G27" s="78"/>
+      <c r="H27" s="78"/>
+      <c r="I27" s="78"/>
     </row>
     <row r="28" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28"/>
-      <c r="B28"/>
-      <c r="C28"/>
-      <c r="D28"/>
-      <c r="E28"/>
-      <c r="F28"/>
-      <c r="G28"/>
-      <c r="H28"/>
-      <c r="I28"/>
+      <c r="B28" s="78"/>
+      <c r="C28" s="78"/>
+      <c r="D28" s="78"/>
+      <c r="E28" s="78"/>
+      <c r="F28" s="78"/>
+      <c r="G28" s="78"/>
+      <c r="H28" s="78"/>
+      <c r="I28" s="78"/>
     </row>
     <row r="29" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29"/>
-      <c r="B29"/>
-      <c r="C29"/>
-      <c r="D29"/>
-      <c r="E29"/>
-      <c r="F29"/>
-      <c r="G29"/>
-      <c r="H29"/>
-      <c r="I29"/>
+      <c r="B29" s="78"/>
+      <c r="C29" s="78"/>
+      <c r="D29" s="78"/>
+      <c r="E29" s="78"/>
+      <c r="F29" s="78"/>
+      <c r="G29" s="78"/>
+      <c r="H29" s="78"/>
+      <c r="I29" s="78"/>
     </row>
     <row r="30" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30"/>
-      <c r="D30"/>
-      <c r="E30"/>
-      <c r="F30"/>
-      <c r="G30"/>
-      <c r="H30"/>
-      <c r="I30"/>
+      <c r="B30" s="78"/>
+      <c r="C30" s="78"/>
+      <c r="D30" s="78"/>
+      <c r="E30" s="78"/>
+      <c r="F30" s="78"/>
+      <c r="G30" s="78"/>
+      <c r="H30" s="78"/>
+      <c r="I30" s="78"/>
     </row>
     <row r="31" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31"/>
-      <c r="B31"/>
-      <c r="C31"/>
-      <c r="D31"/>
-      <c r="E31"/>
-      <c r="F31"/>
-      <c r="G31"/>
-      <c r="H31"/>
-      <c r="I31"/>
+      <c r="B31" s="78"/>
+      <c r="C31" s="78"/>
+      <c r="D31" s="78"/>
+      <c r="E31" s="78"/>
+      <c r="F31" s="78"/>
+      <c r="G31" s="78"/>
+      <c r="H31" s="78"/>
+      <c r="I31" s="78"/>
     </row>
     <row r="32" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32"/>
-      <c r="B32"/>
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32"/>
-      <c r="F32"/>
-      <c r="G32"/>
-      <c r="H32"/>
-      <c r="I32"/>
+      <c r="B32" s="78"/>
+      <c r="C32" s="78"/>
+      <c r="D32" s="78"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="78"/>
+      <c r="G32" s="78"/>
+      <c r="H32" s="78"/>
+      <c r="I32" s="78"/>
     </row>
     <row r="33" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33"/>
-      <c r="B33"/>
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33"/>
-      <c r="F33"/>
-      <c r="G33"/>
-      <c r="H33"/>
-      <c r="I33"/>
+      <c r="B33" s="78"/>
+      <c r="C33" s="78"/>
+      <c r="D33" s="78"/>
+      <c r="E33" s="78"/>
+      <c r="F33" s="78"/>
+      <c r="G33" s="78"/>
+      <c r="H33" s="78"/>
+      <c r="I33" s="78"/>
     </row>
     <row r="34" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34"/>
-      <c r="B34"/>
-      <c r="C34"/>
-      <c r="D34"/>
-      <c r="E34"/>
-      <c r="F34"/>
-      <c r="G34"/>
-      <c r="H34"/>
-      <c r="I34"/>
+      <c r="B34" s="78"/>
+      <c r="C34" s="78"/>
+      <c r="D34" s="78"/>
+      <c r="E34" s="78"/>
+      <c r="F34" s="78"/>
+      <c r="G34" s="78"/>
+      <c r="H34" s="78"/>
+      <c r="I34" s="78"/>
     </row>
     <row r="35" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35"/>
-      <c r="B35"/>
-      <c r="C35"/>
-      <c r="D35"/>
-      <c r="E35"/>
-      <c r="F35"/>
-      <c r="G35"/>
-      <c r="H35"/>
-      <c r="I35"/>
+      <c r="B35" s="78"/>
+      <c r="C35" s="78"/>
+      <c r="D35" s="78"/>
+      <c r="E35" s="78"/>
+      <c r="F35" s="78"/>
+      <c r="G35" s="78"/>
+      <c r="H35" s="78"/>
+      <c r="I35" s="78"/>
     </row>
     <row r="36" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36"/>
-      <c r="B36"/>
-      <c r="C36"/>
-      <c r="D36"/>
-      <c r="E36"/>
-      <c r="F36"/>
-      <c r="G36"/>
-      <c r="H36"/>
-      <c r="I36"/>
+      <c r="B36" s="78"/>
+      <c r="C36" s="78"/>
+      <c r="D36" s="78"/>
+      <c r="E36" s="78"/>
+      <c r="F36" s="78"/>
+      <c r="G36" s="78"/>
+      <c r="H36" s="78"/>
+      <c r="I36" s="78"/>
     </row>
     <row r="37" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37"/>
-      <c r="B37"/>
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37"/>
-      <c r="F37"/>
-      <c r="G37"/>
-      <c r="H37"/>
-      <c r="I37"/>
+      <c r="B37" s="78"/>
+      <c r="C37" s="78"/>
+      <c r="D37" s="78"/>
+      <c r="E37" s="78"/>
+      <c r="F37" s="78"/>
+      <c r="G37" s="78"/>
+      <c r="H37" s="78"/>
+      <c r="I37" s="78"/>
     </row>
     <row r="38" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38"/>
-      <c r="B38"/>
-      <c r="C38"/>
-      <c r="D38"/>
-      <c r="E38"/>
-      <c r="F38"/>
-      <c r="G38"/>
-      <c r="H38"/>
-      <c r="I38"/>
+      <c r="B38" s="78"/>
+      <c r="C38" s="78"/>
+      <c r="D38" s="78"/>
+      <c r="E38" s="78"/>
+      <c r="F38" s="78"/>
+      <c r="G38" s="78"/>
+      <c r="H38" s="78"/>
+      <c r="I38" s="78"/>
     </row>
     <row r="39" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39"/>
-      <c r="B39"/>
-      <c r="C39"/>
-      <c r="D39"/>
-      <c r="E39"/>
-      <c r="F39"/>
-      <c r="G39"/>
-      <c r="H39"/>
-      <c r="I39"/>
+      <c r="B39" s="78"/>
+      <c r="C39" s="78"/>
+      <c r="D39" s="78"/>
+      <c r="E39" s="78"/>
+      <c r="F39" s="78"/>
+      <c r="G39" s="78"/>
+      <c r="H39" s="78"/>
+      <c r="I39" s="78"/>
     </row>
     <row r="40" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40"/>
-      <c r="B40"/>
-      <c r="C40"/>
-      <c r="D40"/>
-      <c r="E40"/>
-      <c r="F40"/>
-      <c r="G40"/>
-      <c r="H40"/>
-      <c r="I40"/>
+      <c r="B40" s="78"/>
+      <c r="C40" s="78"/>
+      <c r="D40" s="78"/>
+      <c r="E40" s="78"/>
+      <c r="F40" s="78"/>
+      <c r="G40" s="78"/>
+      <c r="H40" s="78"/>
+      <c r="I40" s="78"/>
     </row>
     <row r="41" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41"/>
-      <c r="B41"/>
-      <c r="C41"/>
-      <c r="D41"/>
-      <c r="E41"/>
-      <c r="F41"/>
-      <c r="G41"/>
-      <c r="H41"/>
-      <c r="I41"/>
+      <c r="B41" s="78"/>
+      <c r="C41" s="78"/>
+      <c r="D41" s="78"/>
+      <c r="E41" s="78"/>
+      <c r="F41" s="78"/>
+      <c r="G41" s="78"/>
+      <c r="H41" s="78"/>
+      <c r="I41" s="78"/>
     </row>
     <row r="42" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42"/>
-      <c r="B42"/>
-      <c r="C42"/>
-      <c r="D42"/>
-      <c r="E42"/>
-      <c r="F42"/>
-      <c r="G42"/>
-      <c r="H42"/>
-      <c r="I42"/>
+      <c r="B42" s="78"/>
+      <c r="C42" s="78"/>
+      <c r="D42" s="78"/>
+      <c r="E42" s="78"/>
+      <c r="F42" s="78"/>
+      <c r="G42" s="78"/>
+      <c r="H42" s="78"/>
+      <c r="I42" s="78"/>
     </row>
     <row r="43" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43"/>
-      <c r="B43"/>
-      <c r="C43"/>
-      <c r="D43"/>
-      <c r="E43"/>
-      <c r="F43"/>
-      <c r="G43"/>
-      <c r="H43"/>
-      <c r="I43"/>
+      <c r="B43" s="78"/>
+      <c r="C43" s="78"/>
+      <c r="D43" s="78"/>
+      <c r="E43" s="78"/>
+      <c r="F43" s="78"/>
+      <c r="G43" s="78"/>
+      <c r="H43" s="78"/>
+      <c r="I43" s="78"/>
     </row>
     <row r="44" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44"/>
-      <c r="B44"/>
-      <c r="C44"/>
-      <c r="D44"/>
-      <c r="E44"/>
-      <c r="F44"/>
-      <c r="G44"/>
-      <c r="H44"/>
-      <c r="I44"/>
+      <c r="B44" s="78"/>
+      <c r="C44" s="78"/>
+      <c r="D44" s="78"/>
+      <c r="E44" s="78"/>
+      <c r="F44" s="78"/>
+      <c r="G44" s="78"/>
+      <c r="H44" s="78"/>
+      <c r="I44" s="78"/>
     </row>
     <row r="45" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45"/>
-      <c r="B45"/>
-      <c r="C45"/>
-      <c r="D45"/>
-      <c r="E45"/>
-      <c r="F45"/>
-      <c r="G45"/>
-      <c r="H45"/>
-      <c r="I45"/>
+      <c r="B45" s="78"/>
+      <c r="C45" s="78"/>
+      <c r="D45" s="78"/>
+      <c r="E45" s="78"/>
+      <c r="F45" s="78"/>
+      <c r="G45" s="78"/>
+      <c r="H45" s="78"/>
+      <c r="I45" s="78"/>
     </row>
     <row r="46" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46"/>
-      <c r="B46"/>
-      <c r="C46"/>
-      <c r="D46"/>
-      <c r="E46"/>
-      <c r="F46"/>
-      <c r="G46"/>
-      <c r="H46"/>
-      <c r="I46"/>
+      <c r="B46" s="78"/>
+      <c r="C46" s="78"/>
+      <c r="D46" s="78"/>
+      <c r="E46" s="78"/>
+      <c r="F46" s="78"/>
+      <c r="G46" s="78"/>
+      <c r="H46" s="78"/>
+      <c r="I46" s="78"/>
     </row>
     <row r="47" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47"/>
-      <c r="B47"/>
-      <c r="C47"/>
-      <c r="D47"/>
-      <c r="E47"/>
-      <c r="F47"/>
-      <c r="G47"/>
-      <c r="H47"/>
-      <c r="I47"/>
+      <c r="B47" s="78"/>
+      <c r="C47" s="78"/>
+      <c r="D47" s="78"/>
+      <c r="E47" s="78"/>
+      <c r="F47" s="78"/>
+      <c r="G47" s="78"/>
+      <c r="H47" s="78"/>
+      <c r="I47" s="78"/>
     </row>
     <row r="48" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48"/>
-      <c r="B48"/>
-      <c r="C48"/>
-      <c r="D48"/>
-      <c r="E48"/>
-      <c r="F48"/>
-      <c r="G48"/>
-      <c r="H48"/>
-      <c r="I48"/>
+      <c r="B48" s="78"/>
+      <c r="C48" s="78"/>
+      <c r="D48" s="78"/>
+      <c r="E48" s="78"/>
+      <c r="F48" s="78"/>
+      <c r="G48" s="78"/>
+      <c r="H48" s="78"/>
+      <c r="I48" s="78"/>
     </row>
     <row r="49" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49"/>
-      <c r="B49"/>
-      <c r="C49"/>
-      <c r="D49"/>
-      <c r="E49"/>
-      <c r="F49"/>
-      <c r="G49"/>
-      <c r="H49"/>
-      <c r="I49"/>
+      <c r="B49" s="78"/>
+      <c r="C49" s="78"/>
+      <c r="D49" s="78"/>
+      <c r="E49" s="78"/>
+      <c r="F49" s="78"/>
+      <c r="G49" s="78"/>
+      <c r="H49" s="78"/>
+      <c r="I49" s="78"/>
     </row>
     <row r="50" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50"/>
-      <c r="B50"/>
-      <c r="C50"/>
-      <c r="D50"/>
-      <c r="E50"/>
-      <c r="F50"/>
-      <c r="G50"/>
-      <c r="H50"/>
-      <c r="I50"/>
+      <c r="B50" s="78"/>
+      <c r="C50" s="78"/>
+      <c r="D50" s="78"/>
+      <c r="E50" s="78"/>
+      <c r="F50" s="78"/>
+      <c r="G50" s="78"/>
+      <c r="H50" s="78"/>
+      <c r="I50" s="78"/>
     </row>
   </sheetData>
   <sheetProtection insertRows="0" sort="0" autoFilter="0"/>
@@ -2656,56 +2412,88 @@
   <sheetFormatPr defaultColWidth="19.88671875" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.5546875" style="12" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="12" customWidth="1"/>
-    <col min="3" max="3" width="32.44140625" style="12" customWidth="1"/>
-    <col min="4" max="5" width="19.88671875" style="12"/>
-    <col min="6" max="6" width="15.88671875" style="12" customWidth="1"/>
-    <col min="7" max="7" width="23.5546875" style="12" customWidth="1"/>
-    <col min="8" max="8" width="26.88671875" style="12" customWidth="1"/>
-    <col min="9" max="11" width="19.88671875" style="12"/>
+    <col min="2" max="2" width="20.77734375" style="78" customWidth="1"/>
+    <col min="3" max="3" width="32.44140625" style="78" customWidth="1"/>
+    <col min="4" max="5" width="19.88671875" style="78"/>
+    <col min="6" max="6" width="15.88671875" style="78" customWidth="1"/>
+    <col min="7" max="7" width="23.5546875" style="78" customWidth="1"/>
+    <col min="8" max="8" width="26.88671875" style="78" customWidth="1"/>
+    <col min="9" max="9" width="19.88671875" style="78"/>
+    <col min="10" max="11" width="19.88671875" style="12"/>
     <col min="12" max="12" width="19.88671875" style="12" customWidth="1"/>
     <col min="13" max="16384" width="19.88671875" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K1" s="61" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="K1" s="70" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="61"/>
+      <c r="L1" s="70"/>
     </row>
     <row r="2" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K2" s="62" t="s">
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="K2" s="71" t="s">
         <v>55</v>
       </c>
-      <c r="L2" s="62"/>
+      <c r="L2" s="71"/>
     </row>
     <row r="3" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K3" s="62" t="s">
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="K3" s="71" t="s">
         <v>56</v>
       </c>
-      <c r="L3" s="62"/>
+      <c r="L3" s="71"/>
     </row>
     <row r="4" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
       <c r="F4" s="4"/>
-      <c r="K4" s="62" t="s">
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="K4" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="L4" s="62"/>
+      <c r="L4" s="71"/>
     </row>
     <row r="5" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="66" t="s">
+      <c r="B5" s="73" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="66"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="66"/>
-      <c r="F5" s="66"/>
-      <c r="G5" s="66"/>
-      <c r="H5" s="66"/>
-      <c r="I5" s="66"/>
-      <c r="J5" s="66"/>
-      <c r="K5" s="66"/>
-      <c r="L5" s="66"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="73"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="73"/>
+      <c r="J5" s="73"/>
+      <c r="K5" s="73"/>
+      <c r="L5" s="73"/>
     </row>
     <row r="6" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="25"/>
@@ -2715,6 +2503,7 @@
       <c r="F6" s="25"/>
       <c r="G6" s="25"/>
       <c r="H6" s="25"/>
+      <c r="I6" s="12"/>
     </row>
     <row r="7" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="25"/>
@@ -2724,21 +2513,24 @@
       <c r="F7" s="25"/>
       <c r="G7" s="25"/>
       <c r="H7" s="25"/>
+      <c r="I7" s="12"/>
     </row>
     <row r="8" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="60" t="s">
+      <c r="B8" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="60"/>
+      <c r="C8" s="69"/>
       <c r="D8" s="25"/>
       <c r="E8" s="25"/>
       <c r="F8" s="25"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
       <c r="I8" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="J8" s="64"/>
-      <c r="K8" s="64"/>
-      <c r="L8" s="65"/>
+      <c r="J8" s="72"/>
+      <c r="K8" s="72"/>
+      <c r="L8" s="64"/>
     </row>
     <row r="9" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="9" t="s">
@@ -2748,12 +2540,14 @@
       <c r="D9" s="25"/>
       <c r="E9" s="25"/>
       <c r="F9" s="25"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
       <c r="I9" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="J9" s="65"/>
-      <c r="K9" s="67"/>
-      <c r="L9" s="68"/>
+      <c r="J9" s="64"/>
+      <c r="K9" s="65"/>
+      <c r="L9" s="66"/>
     </row>
     <row r="10" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
@@ -2763,12 +2557,14 @@
       <c r="D10" s="25"/>
       <c r="E10" s="25"/>
       <c r="F10" s="25"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
       <c r="I10" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="J10" s="65"/>
-      <c r="K10" s="67"/>
-      <c r="L10" s="68"/>
+      <c r="J10" s="64"/>
+      <c r="K10" s="65"/>
+      <c r="L10" s="66"/>
     </row>
     <row r="11" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="9" t="s">
@@ -2778,12 +2574,14 @@
       <c r="D11" s="25"/>
       <c r="E11" s="25"/>
       <c r="F11" s="25"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
       <c r="I11" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="J11" s="65"/>
-      <c r="K11" s="67"/>
-      <c r="L11" s="68"/>
+      <c r="J11" s="64"/>
+      <c r="K11" s="65"/>
+      <c r="L11" s="66"/>
     </row>
     <row r="12" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="9" t="s">
@@ -2793,12 +2591,14 @@
       <c r="D12" s="25"/>
       <c r="E12" s="25"/>
       <c r="F12" s="25"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
       <c r="I12" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="J12" s="65"/>
-      <c r="K12" s="69"/>
-      <c r="L12" s="70"/>
+      <c r="J12" s="64"/>
+      <c r="K12" s="67"/>
+      <c r="L12" s="68"/>
     </row>
     <row r="13" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="9" t="s">
@@ -2810,6 +2610,7 @@
       <c r="F13" s="25"/>
       <c r="G13" s="25"/>
       <c r="H13" s="25"/>
+      <c r="I13" s="12"/>
     </row>
     <row r="14" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="9" t="s">
@@ -2821,6 +2622,7 @@
       <c r="F14" s="25"/>
       <c r="G14" s="25"/>
       <c r="H14" s="25"/>
+      <c r="I14" s="12"/>
     </row>
     <row r="15" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="25"/>
@@ -2830,6 +2632,7 @@
       <c r="F15" s="25"/>
       <c r="G15" s="25"/>
       <c r="H15" s="25"/>
+      <c r="I15" s="12"/>
     </row>
     <row r="16" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
@@ -2841,6 +2644,7 @@
       <c r="F16" s="25"/>
       <c r="G16" s="25"/>
       <c r="H16" s="25"/>
+      <c r="I16" s="12"/>
     </row>
     <row r="17" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="25" t="s">
@@ -2852,6 +2656,7 @@
       <c r="F17" s="25"/>
       <c r="G17" s="25"/>
       <c r="H17" s="25"/>
+      <c r="I17" s="12"/>
     </row>
     <row r="18" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="25" t="s">
@@ -2863,385 +2668,143 @@
       <c r="F18" s="25"/>
       <c r="G18" s="25"/>
       <c r="H18" s="25"/>
+      <c r="I18" s="12"/>
     </row>
     <row r="19" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="76" t="s">
+      <c r="B19" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="76" t="s">
+      <c r="C19" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="D19" s="76" t="s">
+      <c r="D19" s="49" t="s">
         <v>44</v>
       </c>
-      <c r="E19" s="76" t="s">
+      <c r="E19" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="F19" s="76" t="s">
+      <c r="F19" s="49" t="s">
         <v>46</v>
       </c>
-      <c r="G19" s="76" t="s">
+      <c r="G19" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="H19" s="76" t="s">
+      <c r="H19" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="I19" s="76" t="s">
+      <c r="I19" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="J19" s="76" t="s">
+      <c r="J19" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="K19" s="76" t="s">
+      <c r="K19" s="49" t="s">
         <v>50</v>
       </c>
-      <c r="L19" s="76" t="s">
+      <c r="L19" s="49" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="48"/>
-      <c r="C20" s="48"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="48"/>
-      <c r="H20" s="48"/>
-      <c r="I20" s="48"/>
     </row>
     <row r="21" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21"/>
-      <c r="B21"/>
-      <c r="C21"/>
-      <c r="D21"/>
-      <c r="E21"/>
-      <c r="F21"/>
-      <c r="G21"/>
-      <c r="H21"/>
-      <c r="I21"/>
     </row>
     <row r="22" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22"/>
-      <c r="B22"/>
-      <c r="C22"/>
-      <c r="D22"/>
-      <c r="E22"/>
-      <c r="F22"/>
-      <c r="G22"/>
-      <c r="H22"/>
-      <c r="I22"/>
     </row>
     <row r="23" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23"/>
-      <c r="B23"/>
-      <c r="C23"/>
-      <c r="D23"/>
-      <c r="E23"/>
-      <c r="F23"/>
-      <c r="G23"/>
-      <c r="H23"/>
-      <c r="I23"/>
     </row>
     <row r="24" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24"/>
-      <c r="B24"/>
-      <c r="C24"/>
-      <c r="D24"/>
-      <c r="E24"/>
-      <c r="F24"/>
-      <c r="G24"/>
-      <c r="H24"/>
-      <c r="I24"/>
     </row>
     <row r="25" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25"/>
-      <c r="B25"/>
-      <c r="C25"/>
-      <c r="D25"/>
-      <c r="E25"/>
-      <c r="F25"/>
-      <c r="G25"/>
-      <c r="H25"/>
-      <c r="I25"/>
     </row>
     <row r="26" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26"/>
-      <c r="B26"/>
-      <c r="C26"/>
-      <c r="D26"/>
-      <c r="E26"/>
-      <c r="F26"/>
-      <c r="G26"/>
-      <c r="H26"/>
-      <c r="I26"/>
     </row>
     <row r="27" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27"/>
-      <c r="B27"/>
-      <c r="C27"/>
-      <c r="D27"/>
-      <c r="E27"/>
-      <c r="F27"/>
-      <c r="G27"/>
-      <c r="H27"/>
-      <c r="I27"/>
     </row>
     <row r="28" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28"/>
-      <c r="B28"/>
-      <c r="C28"/>
-      <c r="D28"/>
-      <c r="E28"/>
-      <c r="F28"/>
-      <c r="G28"/>
-      <c r="H28"/>
-      <c r="I28"/>
     </row>
     <row r="29" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29"/>
-      <c r="B29"/>
-      <c r="C29"/>
-      <c r="D29"/>
-      <c r="E29"/>
-      <c r="F29"/>
-      <c r="G29"/>
-      <c r="H29"/>
-      <c r="I29"/>
     </row>
     <row r="30" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30"/>
-      <c r="D30"/>
-      <c r="E30"/>
-      <c r="F30"/>
-      <c r="G30"/>
-      <c r="H30"/>
-      <c r="I30"/>
     </row>
     <row r="31" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31"/>
-      <c r="B31"/>
-      <c r="C31"/>
-      <c r="D31"/>
-      <c r="E31"/>
-      <c r="F31"/>
-      <c r="G31"/>
-      <c r="H31"/>
-      <c r="I31"/>
     </row>
     <row r="32" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32"/>
-      <c r="B32"/>
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32"/>
-      <c r="F32"/>
-      <c r="G32"/>
-      <c r="H32"/>
-      <c r="I32"/>
-    </row>
-    <row r="33" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="33" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33"/>
-      <c r="B33"/>
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33"/>
-      <c r="F33"/>
-      <c r="G33"/>
-      <c r="H33"/>
-      <c r="I33"/>
-    </row>
-    <row r="34" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="34" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34"/>
-      <c r="B34"/>
-      <c r="C34"/>
-      <c r="D34"/>
-      <c r="E34"/>
-      <c r="F34"/>
-      <c r="G34"/>
-      <c r="H34"/>
-      <c r="I34"/>
-    </row>
-    <row r="35" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="35" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35"/>
-      <c r="B35"/>
-      <c r="C35"/>
-      <c r="D35"/>
-      <c r="E35"/>
-      <c r="F35"/>
-      <c r="G35"/>
-      <c r="H35"/>
-      <c r="I35"/>
-    </row>
-    <row r="36" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="36" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36"/>
-      <c r="B36"/>
-      <c r="C36"/>
-      <c r="D36"/>
-      <c r="E36"/>
-      <c r="F36"/>
-      <c r="G36"/>
-      <c r="H36"/>
-      <c r="I36"/>
-    </row>
-    <row r="37" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="37" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37"/>
-      <c r="B37"/>
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37"/>
-      <c r="F37"/>
-      <c r="G37"/>
-      <c r="H37"/>
-      <c r="I37"/>
-    </row>
-    <row r="38" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="38" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38"/>
-      <c r="B38"/>
-      <c r="C38"/>
-      <c r="D38"/>
-      <c r="E38"/>
-      <c r="F38"/>
-      <c r="G38"/>
-      <c r="H38"/>
-      <c r="I38"/>
-    </row>
-    <row r="39" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39"/>
-      <c r="B39"/>
-      <c r="C39"/>
-      <c r="D39"/>
-      <c r="E39"/>
-      <c r="F39"/>
-      <c r="G39"/>
-      <c r="H39"/>
-      <c r="I39"/>
-    </row>
-    <row r="40" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40"/>
-      <c r="B40"/>
-      <c r="C40"/>
-      <c r="D40"/>
-      <c r="E40"/>
-      <c r="F40"/>
-      <c r="G40"/>
-      <c r="H40"/>
-      <c r="I40"/>
-    </row>
-    <row r="41" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41"/>
-      <c r="B41"/>
-      <c r="C41"/>
-      <c r="D41"/>
-      <c r="E41"/>
-      <c r="F41"/>
-      <c r="G41"/>
-      <c r="H41"/>
-      <c r="I41"/>
-    </row>
-    <row r="42" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42"/>
-      <c r="B42"/>
-      <c r="C42"/>
-      <c r="D42"/>
-      <c r="E42"/>
-      <c r="F42"/>
-      <c r="G42"/>
-      <c r="H42"/>
-      <c r="I42"/>
-    </row>
-    <row r="43" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43"/>
-      <c r="B43"/>
-      <c r="C43"/>
-      <c r="D43"/>
-      <c r="E43"/>
-      <c r="F43"/>
-      <c r="G43"/>
-      <c r="H43"/>
-      <c r="I43"/>
-    </row>
-    <row r="44" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44"/>
-      <c r="B44"/>
-      <c r="C44"/>
-      <c r="D44"/>
-      <c r="E44"/>
-      <c r="F44"/>
-      <c r="G44"/>
-      <c r="H44"/>
-      <c r="I44"/>
-    </row>
-    <row r="45" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="45" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45"/>
-      <c r="B45"/>
-      <c r="C45"/>
-      <c r="D45"/>
-      <c r="E45"/>
-      <c r="F45"/>
-      <c r="G45"/>
-      <c r="H45"/>
-      <c r="I45"/>
-    </row>
-    <row r="46" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="46" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46"/>
-      <c r="B46"/>
-      <c r="C46"/>
-      <c r="D46"/>
-      <c r="E46"/>
-      <c r="F46"/>
-      <c r="G46"/>
-      <c r="H46"/>
-      <c r="I46"/>
-    </row>
-    <row r="47" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47"/>
-      <c r="B47"/>
-      <c r="C47"/>
-      <c r="D47"/>
-      <c r="E47"/>
-      <c r="F47"/>
-      <c r="G47"/>
-      <c r="H47"/>
-      <c r="I47"/>
-    </row>
-    <row r="48" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48"/>
-      <c r="B48"/>
-      <c r="C48"/>
-      <c r="D48"/>
-      <c r="E48"/>
-      <c r="F48"/>
-      <c r="G48"/>
-      <c r="H48"/>
-      <c r="I48"/>
-    </row>
-    <row r="49" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="49" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49"/>
-      <c r="B49"/>
-      <c r="C49"/>
-      <c r="D49"/>
-      <c r="E49"/>
-      <c r="F49"/>
-      <c r="G49"/>
-      <c r="H49"/>
-      <c r="I49"/>
-    </row>
-    <row r="50" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="50" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50"/>
-      <c r="B50"/>
-      <c r="C50"/>
-      <c r="D50"/>
-      <c r="E50"/>
-      <c r="F50"/>
-      <c r="G50"/>
-      <c r="H50"/>
-      <c r="I50"/>
     </row>
   </sheetData>
   <sheetProtection insertRows="0" sort="0" autoFilter="0"/>
   <mergeCells count="15">
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="I8:L8"/>
+    <mergeCell ref="B5:L5"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="I10:J10"/>
     <mergeCell ref="I11:J11"/>
@@ -3250,13 +2813,6 @@
     <mergeCell ref="K10:L10"/>
     <mergeCell ref="K11:L11"/>
     <mergeCell ref="K12:L12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="I8:L8"/>
-    <mergeCell ref="B5:L5"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date" error="Please enter a valid date" sqref="C13:C14" xr:uid="{FA1C3AB6-2DE1-499E-8DD7-9A28238B7787}">
@@ -3280,47 +2836,48 @@
   <sheetFormatPr defaultColWidth="19.88671875" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.5546875" style="12" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="12" customWidth="1"/>
-    <col min="3" max="3" width="32.44140625" style="12" customWidth="1"/>
-    <col min="4" max="5" width="19.88671875" style="12"/>
-    <col min="6" max="6" width="15.88671875" style="12" customWidth="1"/>
-    <col min="7" max="7" width="23.5546875" style="12" customWidth="1"/>
-    <col min="8" max="8" width="26.88671875" style="12" customWidth="1"/>
-    <col min="9" max="16384" width="19.88671875" style="12"/>
+    <col min="2" max="2" width="20.77734375" style="78" customWidth="1"/>
+    <col min="3" max="3" width="32.44140625" style="78" customWidth="1"/>
+    <col min="4" max="5" width="19.88671875" style="78"/>
+    <col min="6" max="6" width="15.88671875" style="78" customWidth="1"/>
+    <col min="7" max="7" width="23.5546875" style="78" customWidth="1"/>
+    <col min="8" max="8" width="26.88671875" style="78" customWidth="1"/>
+    <col min="9" max="9" width="19.88671875" style="78"/>
+    <col min="10" max="16384" width="19.88671875" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H2" s="13" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H3" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H4" s="13" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="57" t="s">
+    <row r="5" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-    </row>
-    <row r="6" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+    </row>
+    <row r="6" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="25"/>
       <c r="C6" s="25"/>
       <c r="D6" s="25"/>
@@ -3329,7 +2886,7 @@
       <c r="G6" s="25"/>
       <c r="H6" s="25"/>
     </row>
-    <row r="7" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="25"/>
       <c r="C7" s="25"/>
       <c r="D7" s="25"/>
@@ -3338,20 +2895,20 @@
       <c r="G7" s="25"/>
       <c r="H7" s="25"/>
     </row>
-    <row r="8" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="71" t="s">
+    <row r="8" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="71"/>
+      <c r="C8" s="74"/>
       <c r="D8" s="25"/>
       <c r="E8" s="25"/>
       <c r="F8" s="25"/>
-      <c r="G8" s="71" t="s">
+      <c r="G8" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="H8" s="71"/>
-    </row>
-    <row r="9" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H8" s="74"/>
+    </row>
+    <row r="9" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
         <v>2</v>
       </c>
@@ -3364,7 +2921,7 @@
       </c>
       <c r="H9" s="37"/>
     </row>
-    <row r="10" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="6" t="s">
         <v>3</v>
       </c>
@@ -3377,7 +2934,7 @@
       </c>
       <c r="H10" s="37"/>
     </row>
-    <row r="11" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="6" t="s">
         <v>4</v>
       </c>
@@ -3390,7 +2947,7 @@
       </c>
       <c r="H11" s="37"/>
     </row>
-    <row r="12" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="6" t="s">
         <v>6</v>
       </c>
@@ -3403,7 +2960,7 @@
       </c>
       <c r="H12" s="39"/>
     </row>
-    <row r="13" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="6" t="s">
         <v>5</v>
       </c>
@@ -3414,7 +2971,7 @@
       <c r="G13" s="25"/>
       <c r="H13" s="25"/>
     </row>
-    <row r="14" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="6" t="s">
         <v>22</v>
       </c>
@@ -3425,7 +2982,7 @@
       <c r="G14" s="25"/>
       <c r="H14" s="25"/>
     </row>
-    <row r="15" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="25"/>
       <c r="C15" s="25"/>
       <c r="D15" s="25"/>
@@ -3434,7 +2991,7 @@
       <c r="G15" s="25"/>
       <c r="H15" s="25"/>
     </row>
-    <row r="16" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:8" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="40" t="s">
         <v>59</v>
       </c>
@@ -3455,6 +3012,7 @@
       <c r="F17" s="25"/>
       <c r="G17" s="25"/>
       <c r="H17" s="25"/>
+      <c r="I17" s="12"/>
     </row>
     <row r="18" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="36" t="s">
@@ -3466,369 +3024,120 @@
       <c r="F18" s="25"/>
       <c r="G18" s="25"/>
       <c r="H18" s="25"/>
+      <c r="I18" s="12"/>
     </row>
     <row r="19" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="77" t="s">
+      <c r="B19" s="50" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="77" t="s">
+      <c r="C19" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="77" t="s">
+      <c r="D19" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="E19" s="77" t="s">
+      <c r="E19" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="F19" s="77" t="s">
+      <c r="F19" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="77" t="s">
+      <c r="G19" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="H19" s="77" t="s">
+      <c r="H19" s="50" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="48"/>
-      <c r="C20" s="48"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="48"/>
-      <c r="H20" s="48"/>
-      <c r="I20" s="48"/>
     </row>
     <row r="21" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21"/>
-      <c r="B21"/>
-      <c r="C21"/>
-      <c r="D21"/>
-      <c r="E21"/>
-      <c r="F21"/>
-      <c r="G21"/>
-      <c r="H21"/>
-      <c r="I21"/>
     </row>
     <row r="22" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22"/>
-      <c r="B22"/>
-      <c r="C22"/>
-      <c r="D22"/>
-      <c r="E22"/>
-      <c r="F22"/>
-      <c r="G22"/>
-      <c r="H22"/>
-      <c r="I22"/>
     </row>
     <row r="23" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23"/>
-      <c r="B23"/>
-      <c r="C23"/>
-      <c r="D23"/>
-      <c r="E23"/>
-      <c r="F23"/>
-      <c r="G23"/>
-      <c r="H23"/>
-      <c r="I23"/>
     </row>
     <row r="24" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24"/>
-      <c r="B24"/>
-      <c r="C24"/>
-      <c r="D24"/>
-      <c r="E24"/>
-      <c r="F24"/>
-      <c r="G24"/>
-      <c r="H24"/>
-      <c r="I24"/>
     </row>
     <row r="25" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25"/>
-      <c r="B25"/>
-      <c r="C25"/>
-      <c r="D25"/>
-      <c r="E25"/>
-      <c r="F25"/>
-      <c r="G25"/>
-      <c r="H25"/>
-      <c r="I25"/>
     </row>
     <row r="26" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26"/>
-      <c r="B26"/>
-      <c r="C26"/>
-      <c r="D26"/>
-      <c r="E26"/>
-      <c r="F26"/>
-      <c r="G26"/>
-      <c r="H26"/>
-      <c r="I26"/>
     </row>
     <row r="27" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27"/>
-      <c r="B27"/>
-      <c r="C27"/>
-      <c r="D27"/>
-      <c r="E27"/>
-      <c r="F27"/>
-      <c r="G27"/>
-      <c r="H27"/>
-      <c r="I27"/>
     </row>
     <row r="28" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28"/>
-      <c r="B28"/>
-      <c r="C28"/>
-      <c r="D28"/>
-      <c r="E28"/>
-      <c r="F28"/>
-      <c r="G28"/>
-      <c r="H28"/>
-      <c r="I28"/>
     </row>
     <row r="29" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29"/>
-      <c r="B29"/>
-      <c r="C29"/>
-      <c r="D29"/>
-      <c r="E29"/>
-      <c r="F29"/>
-      <c r="G29"/>
-      <c r="H29"/>
-      <c r="I29"/>
     </row>
     <row r="30" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30"/>
-      <c r="D30"/>
-      <c r="E30"/>
-      <c r="F30"/>
-      <c r="G30"/>
-      <c r="H30"/>
-      <c r="I30"/>
     </row>
     <row r="31" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31"/>
-      <c r="B31"/>
-      <c r="C31"/>
-      <c r="D31"/>
-      <c r="E31"/>
-      <c r="F31"/>
-      <c r="G31"/>
-      <c r="H31"/>
-      <c r="I31"/>
     </row>
     <row r="32" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32"/>
-      <c r="B32"/>
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32"/>
-      <c r="F32"/>
-      <c r="G32"/>
-      <c r="H32"/>
-      <c r="I32"/>
-    </row>
-    <row r="33" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="33" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33"/>
-      <c r="B33"/>
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33"/>
-      <c r="F33"/>
-      <c r="G33"/>
-      <c r="H33"/>
-      <c r="I33"/>
-    </row>
-    <row r="34" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="34" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34"/>
-      <c r="B34"/>
-      <c r="C34"/>
-      <c r="D34"/>
-      <c r="E34"/>
-      <c r="F34"/>
-      <c r="G34"/>
-      <c r="H34"/>
-      <c r="I34"/>
-    </row>
-    <row r="35" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="35" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35"/>
-      <c r="B35"/>
-      <c r="C35"/>
-      <c r="D35"/>
-      <c r="E35"/>
-      <c r="F35"/>
-      <c r="G35"/>
-      <c r="H35"/>
-      <c r="I35"/>
-    </row>
-    <row r="36" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="36" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36"/>
-      <c r="B36"/>
-      <c r="C36"/>
-      <c r="D36"/>
-      <c r="E36"/>
-      <c r="F36"/>
-      <c r="G36"/>
-      <c r="H36"/>
-      <c r="I36"/>
-    </row>
-    <row r="37" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="37" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37"/>
-      <c r="B37"/>
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37"/>
-      <c r="F37"/>
-      <c r="G37"/>
-      <c r="H37"/>
-      <c r="I37"/>
-    </row>
-    <row r="38" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="38" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38"/>
-      <c r="B38"/>
-      <c r="C38"/>
-      <c r="D38"/>
-      <c r="E38"/>
-      <c r="F38"/>
-      <c r="G38"/>
-      <c r="H38"/>
-      <c r="I38"/>
-    </row>
-    <row r="39" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39"/>
-      <c r="B39"/>
-      <c r="C39"/>
-      <c r="D39"/>
-      <c r="E39"/>
-      <c r="F39"/>
-      <c r="G39"/>
-      <c r="H39"/>
-      <c r="I39"/>
-    </row>
-    <row r="40" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40"/>
-      <c r="B40"/>
-      <c r="C40"/>
-      <c r="D40"/>
-      <c r="E40"/>
-      <c r="F40"/>
-      <c r="G40"/>
-      <c r="H40"/>
-      <c r="I40"/>
-    </row>
-    <row r="41" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41"/>
-      <c r="B41"/>
-      <c r="C41"/>
-      <c r="D41"/>
-      <c r="E41"/>
-      <c r="F41"/>
-      <c r="G41"/>
-      <c r="H41"/>
-      <c r="I41"/>
-    </row>
-    <row r="42" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42"/>
-      <c r="B42"/>
-      <c r="C42"/>
-      <c r="D42"/>
-      <c r="E42"/>
-      <c r="F42"/>
-      <c r="G42"/>
-      <c r="H42"/>
-      <c r="I42"/>
-    </row>
-    <row r="43" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43"/>
-      <c r="B43"/>
-      <c r="C43"/>
-      <c r="D43"/>
-      <c r="E43"/>
-      <c r="F43"/>
-      <c r="G43"/>
-      <c r="H43"/>
-      <c r="I43"/>
-    </row>
-    <row r="44" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44"/>
-      <c r="B44"/>
-      <c r="C44"/>
-      <c r="D44"/>
-      <c r="E44"/>
-      <c r="F44"/>
-      <c r="G44"/>
-      <c r="H44"/>
-      <c r="I44"/>
-    </row>
-    <row r="45" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="45" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45"/>
-      <c r="B45"/>
-      <c r="C45"/>
-      <c r="D45"/>
-      <c r="E45"/>
-      <c r="F45"/>
-      <c r="G45"/>
-      <c r="H45"/>
-      <c r="I45"/>
-    </row>
-    <row r="46" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="46" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46"/>
-      <c r="B46"/>
-      <c r="C46"/>
-      <c r="D46"/>
-      <c r="E46"/>
-      <c r="F46"/>
-      <c r="G46"/>
-      <c r="H46"/>
-      <c r="I46"/>
-    </row>
-    <row r="47" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47"/>
-      <c r="B47"/>
-      <c r="C47"/>
-      <c r="D47"/>
-      <c r="E47"/>
-      <c r="F47"/>
-      <c r="G47"/>
-      <c r="H47"/>
-      <c r="I47"/>
-    </row>
-    <row r="48" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48"/>
-      <c r="B48"/>
-      <c r="C48"/>
-      <c r="D48"/>
-      <c r="E48"/>
-      <c r="F48"/>
-      <c r="G48"/>
-      <c r="H48"/>
-      <c r="I48"/>
-    </row>
-    <row r="49" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="49" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49"/>
-      <c r="B49"/>
-      <c r="C49"/>
-      <c r="D49"/>
-      <c r="E49"/>
-      <c r="F49"/>
-      <c r="G49"/>
-      <c r="H49"/>
-      <c r="I49"/>
-    </row>
-    <row r="50" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="50" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50"/>
-      <c r="B50"/>
-      <c r="C50"/>
-      <c r="D50"/>
-      <c r="E50"/>
-      <c r="F50"/>
-      <c r="G50"/>
-      <c r="H50"/>
-      <c r="I50"/>
     </row>
   </sheetData>
   <sheetProtection insertRows="0" sort="0" autoFilter="0"/>
@@ -3859,66 +3168,119 @@
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" style="25" customWidth="1"/>
-    <col min="2" max="2" width="29" style="25" customWidth="1"/>
-    <col min="3" max="4" width="29.6640625" style="25" customWidth="1"/>
-    <col min="5" max="5" width="21.109375" style="25" customWidth="1"/>
-    <col min="6" max="6" width="24.6640625" style="25" customWidth="1"/>
-    <col min="7" max="7" width="23.5546875" style="25" customWidth="1"/>
-    <col min="8" max="8" width="32.33203125" style="25" customWidth="1"/>
-    <col min="9" max="9" width="43.77734375" style="25" customWidth="1"/>
+    <col min="2" max="2" width="29" style="13" customWidth="1"/>
+    <col min="3" max="4" width="29.6640625" style="13" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" style="13" customWidth="1"/>
+    <col min="6" max="6" width="24.6640625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="23.5546875" style="13" customWidth="1"/>
+    <col min="8" max="8" width="32.33203125" style="13" customWidth="1"/>
+    <col min="9" max="9" width="43.77734375" style="13" customWidth="1"/>
     <col min="10" max="16384" width="8.88671875" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
       <c r="I1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="2" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
       <c r="I2" s="13" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="3" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
       <c r="I3" s="13" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="4" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
       <c r="I4" s="13" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="5" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="57" t="s">
+      <c r="B5" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="60"/>
     </row>
     <row r="6" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="25"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
       <c r="E6" s="41"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
+    </row>
+    <row r="7" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="25"/>
     </row>
     <row r="8" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="72" t="s">
+      <c r="B8" s="75" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="72"/>
-      <c r="H8" s="73" t="s">
+      <c r="C8" s="75"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="I8" s="74"/>
+      <c r="I8" s="77"/>
     </row>
     <row r="9" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="42" t="s">
         <v>2</v>
       </c>
       <c r="C9" s="43"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
       <c r="H9" s="42" t="s">
         <v>20</v>
       </c>
@@ -3929,6 +3291,10 @@
         <v>3</v>
       </c>
       <c r="C10" s="43"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
       <c r="H10" s="42" t="s">
         <v>3</v>
       </c>
@@ -3939,6 +3305,10 @@
         <v>4</v>
       </c>
       <c r="C11" s="43"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
       <c r="H11" s="42" t="s">
         <v>5</v>
       </c>
@@ -3949,6 +3319,10 @@
         <v>6</v>
       </c>
       <c r="C12" s="45"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
       <c r="H12" s="42" t="s">
         <v>21</v>
       </c>
@@ -3959,393 +3333,426 @@
         <v>5</v>
       </c>
       <c r="C13" s="43"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="25"/>
+      <c r="H13" s="25"/>
+      <c r="I13" s="25"/>
     </row>
     <row r="14" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="42" t="s">
         <v>22</v>
       </c>
       <c r="C14" s="43"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="25"/>
+    </row>
+    <row r="15" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
     </row>
     <row r="16" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="34" t="s">
         <v>60</v>
       </c>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
     </row>
     <row r="17" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="47" t="s">
         <v>23</v>
       </c>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
     </row>
     <row r="18" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="47" t="s">
         <v>24</v>
       </c>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
     </row>
     <row r="19" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="78" t="s">
+      <c r="B19" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="78" t="s">
+      <c r="C19" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="78" t="s">
+      <c r="D19" s="51" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="78" t="s">
+      <c r="E19" s="51" t="s">
         <v>32</v>
       </c>
-      <c r="F19" s="78" t="s">
+      <c r="F19" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="G19" s="78" t="s">
+      <c r="G19" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="H19" s="78" t="s">
+      <c r="H19" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="I19" s="78" t="s">
+      <c r="I19" s="51" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="36"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="36"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="36"/>
-      <c r="I20" s="36"/>
     </row>
     <row r="21" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21"/>
-      <c r="B21"/>
-      <c r="C21"/>
-      <c r="D21"/>
-      <c r="E21"/>
-      <c r="F21"/>
-      <c r="G21"/>
-      <c r="H21"/>
-      <c r="I21"/>
+      <c r="B21" s="78"/>
+      <c r="C21" s="78"/>
+      <c r="D21" s="78"/>
+      <c r="E21" s="78"/>
+      <c r="F21" s="78"/>
+      <c r="G21" s="78"/>
+      <c r="H21" s="78"/>
+      <c r="I21" s="78"/>
     </row>
     <row r="22" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22"/>
-      <c r="B22"/>
-      <c r="C22"/>
-      <c r="D22"/>
-      <c r="E22"/>
-      <c r="F22"/>
-      <c r="G22"/>
-      <c r="H22"/>
-      <c r="I22"/>
+      <c r="B22" s="78"/>
+      <c r="C22" s="78"/>
+      <c r="D22" s="78"/>
+      <c r="E22" s="78"/>
+      <c r="F22" s="78"/>
+      <c r="G22" s="78"/>
+      <c r="H22" s="78"/>
+      <c r="I22" s="78"/>
     </row>
     <row r="23" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23"/>
-      <c r="B23"/>
-      <c r="C23"/>
-      <c r="D23"/>
-      <c r="E23"/>
-      <c r="F23"/>
-      <c r="G23"/>
-      <c r="H23"/>
-      <c r="I23"/>
+      <c r="B23" s="78"/>
+      <c r="C23" s="78"/>
+      <c r="D23" s="78"/>
+      <c r="E23" s="78"/>
+      <c r="F23" s="78"/>
+      <c r="G23" s="78"/>
+      <c r="H23" s="78"/>
+      <c r="I23" s="78"/>
     </row>
     <row r="24" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24"/>
-      <c r="B24"/>
-      <c r="C24"/>
-      <c r="D24"/>
-      <c r="E24"/>
-      <c r="F24"/>
-      <c r="G24"/>
-      <c r="H24"/>
-      <c r="I24"/>
+      <c r="B24" s="78"/>
+      <c r="C24" s="78"/>
+      <c r="D24" s="78"/>
+      <c r="E24" s="78"/>
+      <c r="F24" s="78"/>
+      <c r="G24" s="78"/>
+      <c r="H24" s="78"/>
+      <c r="I24" s="78"/>
     </row>
     <row r="25" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25"/>
-      <c r="B25"/>
-      <c r="C25"/>
-      <c r="D25"/>
-      <c r="E25"/>
-      <c r="F25"/>
-      <c r="G25"/>
-      <c r="H25"/>
-      <c r="I25"/>
+      <c r="B25" s="78"/>
+      <c r="C25" s="78"/>
+      <c r="D25" s="78"/>
+      <c r="E25" s="78"/>
+      <c r="F25" s="78"/>
+      <c r="G25" s="78"/>
+      <c r="H25" s="78"/>
+      <c r="I25" s="78"/>
     </row>
     <row r="26" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26"/>
-      <c r="B26"/>
-      <c r="C26"/>
-      <c r="D26"/>
-      <c r="E26"/>
-      <c r="F26"/>
-      <c r="G26"/>
-      <c r="H26"/>
-      <c r="I26"/>
+      <c r="B26" s="78"/>
+      <c r="C26" s="78"/>
+      <c r="D26" s="78"/>
+      <c r="E26" s="78"/>
+      <c r="F26" s="78"/>
+      <c r="G26" s="78"/>
+      <c r="H26" s="78"/>
+      <c r="I26" s="78"/>
     </row>
     <row r="27" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27"/>
-      <c r="B27"/>
-      <c r="C27"/>
-      <c r="D27"/>
-      <c r="E27"/>
-      <c r="F27"/>
-      <c r="G27"/>
-      <c r="H27"/>
-      <c r="I27"/>
+      <c r="B27" s="78"/>
+      <c r="C27" s="78"/>
+      <c r="D27" s="78"/>
+      <c r="E27" s="78"/>
+      <c r="F27" s="78"/>
+      <c r="G27" s="78"/>
+      <c r="H27" s="78"/>
+      <c r="I27" s="78"/>
     </row>
     <row r="28" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28"/>
-      <c r="B28"/>
-      <c r="C28"/>
-      <c r="D28"/>
-      <c r="E28"/>
-      <c r="F28"/>
-      <c r="G28"/>
-      <c r="H28"/>
-      <c r="I28"/>
+      <c r="B28" s="78"/>
+      <c r="C28" s="78"/>
+      <c r="D28" s="78"/>
+      <c r="E28" s="78"/>
+      <c r="F28" s="78"/>
+      <c r="G28" s="78"/>
+      <c r="H28" s="78"/>
+      <c r="I28" s="78"/>
     </row>
     <row r="29" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29"/>
-      <c r="B29"/>
-      <c r="C29"/>
-      <c r="D29"/>
-      <c r="E29"/>
-      <c r="F29"/>
-      <c r="G29"/>
-      <c r="H29"/>
-      <c r="I29"/>
+      <c r="B29" s="78"/>
+      <c r="C29" s="78"/>
+      <c r="D29" s="78"/>
+      <c r="E29" s="78"/>
+      <c r="F29" s="78"/>
+      <c r="G29" s="78"/>
+      <c r="H29" s="78"/>
+      <c r="I29" s="78"/>
     </row>
     <row r="30" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30"/>
-      <c r="D30"/>
-      <c r="E30"/>
-      <c r="F30"/>
-      <c r="G30"/>
-      <c r="H30"/>
-      <c r="I30"/>
+      <c r="B30" s="78"/>
+      <c r="C30" s="78"/>
+      <c r="D30" s="78"/>
+      <c r="E30" s="78"/>
+      <c r="F30" s="78"/>
+      <c r="G30" s="78"/>
+      <c r="H30" s="78"/>
+      <c r="I30" s="78"/>
     </row>
     <row r="31" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31"/>
-      <c r="B31"/>
-      <c r="C31"/>
-      <c r="D31"/>
-      <c r="E31"/>
-      <c r="F31"/>
-      <c r="G31"/>
-      <c r="H31"/>
-      <c r="I31"/>
+      <c r="B31" s="78"/>
+      <c r="C31" s="78"/>
+      <c r="D31" s="78"/>
+      <c r="E31" s="78"/>
+      <c r="F31" s="78"/>
+      <c r="G31" s="78"/>
+      <c r="H31" s="78"/>
+      <c r="I31" s="78"/>
     </row>
     <row r="32" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32"/>
-      <c r="B32"/>
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32"/>
-      <c r="F32"/>
-      <c r="G32"/>
-      <c r="H32"/>
-      <c r="I32"/>
+      <c r="B32" s="78"/>
+      <c r="C32" s="78"/>
+      <c r="D32" s="78"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="78"/>
+      <c r="G32" s="78"/>
+      <c r="H32" s="78"/>
+      <c r="I32" s="78"/>
     </row>
     <row r="33" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33"/>
-      <c r="B33"/>
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33"/>
-      <c r="F33"/>
-      <c r="G33"/>
-      <c r="H33"/>
-      <c r="I33"/>
+      <c r="B33" s="78"/>
+      <c r="C33" s="78"/>
+      <c r="D33" s="78"/>
+      <c r="E33" s="78"/>
+      <c r="F33" s="78"/>
+      <c r="G33" s="78"/>
+      <c r="H33" s="78"/>
+      <c r="I33" s="78"/>
     </row>
     <row r="34" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34"/>
-      <c r="B34"/>
-      <c r="C34"/>
-      <c r="D34"/>
-      <c r="E34"/>
-      <c r="F34"/>
-      <c r="G34"/>
-      <c r="H34"/>
-      <c r="I34"/>
+      <c r="B34" s="78"/>
+      <c r="C34" s="78"/>
+      <c r="D34" s="78"/>
+      <c r="E34" s="78"/>
+      <c r="F34" s="78"/>
+      <c r="G34" s="78"/>
+      <c r="H34" s="78"/>
+      <c r="I34" s="78"/>
     </row>
     <row r="35" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35"/>
-      <c r="B35"/>
-      <c r="C35"/>
-      <c r="D35"/>
-      <c r="E35"/>
-      <c r="F35"/>
-      <c r="G35"/>
-      <c r="H35"/>
-      <c r="I35"/>
+      <c r="B35" s="78"/>
+      <c r="C35" s="78"/>
+      <c r="D35" s="78"/>
+      <c r="E35" s="78"/>
+      <c r="F35" s="78"/>
+      <c r="G35" s="78"/>
+      <c r="H35" s="78"/>
+      <c r="I35" s="78"/>
     </row>
     <row r="36" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36"/>
-      <c r="B36"/>
-      <c r="C36"/>
-      <c r="D36"/>
-      <c r="E36"/>
-      <c r="F36"/>
-      <c r="G36"/>
-      <c r="H36"/>
-      <c r="I36"/>
+      <c r="B36" s="78"/>
+      <c r="C36" s="78"/>
+      <c r="D36" s="78"/>
+      <c r="E36" s="78"/>
+      <c r="F36" s="78"/>
+      <c r="G36" s="78"/>
+      <c r="H36" s="78"/>
+      <c r="I36" s="78"/>
     </row>
     <row r="37" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37"/>
-      <c r="B37"/>
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37"/>
-      <c r="F37"/>
-      <c r="G37"/>
-      <c r="H37"/>
-      <c r="I37"/>
+      <c r="B37" s="78"/>
+      <c r="C37" s="78"/>
+      <c r="D37" s="78"/>
+      <c r="E37" s="78"/>
+      <c r="F37" s="78"/>
+      <c r="G37" s="78"/>
+      <c r="H37" s="78"/>
+      <c r="I37" s="78"/>
     </row>
     <row r="38" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38"/>
-      <c r="B38"/>
-      <c r="C38"/>
-      <c r="D38"/>
-      <c r="E38"/>
-      <c r="F38"/>
-      <c r="G38"/>
-      <c r="H38"/>
-      <c r="I38"/>
+      <c r="B38" s="78"/>
+      <c r="C38" s="78"/>
+      <c r="D38" s="78"/>
+      <c r="E38" s="78"/>
+      <c r="F38" s="78"/>
+      <c r="G38" s="78"/>
+      <c r="H38" s="78"/>
+      <c r="I38" s="78"/>
     </row>
     <row r="39" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39"/>
-      <c r="B39"/>
-      <c r="C39"/>
-      <c r="D39"/>
-      <c r="E39"/>
-      <c r="F39"/>
-      <c r="G39"/>
-      <c r="H39"/>
-      <c r="I39"/>
+      <c r="B39" s="78"/>
+      <c r="C39" s="78"/>
+      <c r="D39" s="78"/>
+      <c r="E39" s="78"/>
+      <c r="F39" s="78"/>
+      <c r="G39" s="78"/>
+      <c r="H39" s="78"/>
+      <c r="I39" s="78"/>
     </row>
     <row r="40" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40"/>
-      <c r="B40"/>
-      <c r="C40"/>
-      <c r="D40"/>
-      <c r="E40"/>
-      <c r="F40"/>
-      <c r="G40"/>
-      <c r="H40"/>
-      <c r="I40"/>
+      <c r="B40" s="78"/>
+      <c r="C40" s="78"/>
+      <c r="D40" s="78"/>
+      <c r="E40" s="78"/>
+      <c r="F40" s="78"/>
+      <c r="G40" s="78"/>
+      <c r="H40" s="78"/>
+      <c r="I40" s="78"/>
     </row>
     <row r="41" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41"/>
-      <c r="B41"/>
-      <c r="C41"/>
-      <c r="D41"/>
-      <c r="E41"/>
-      <c r="F41"/>
-      <c r="G41"/>
-      <c r="H41"/>
-      <c r="I41"/>
+      <c r="B41" s="78"/>
+      <c r="C41" s="78"/>
+      <c r="D41" s="78"/>
+      <c r="E41" s="78"/>
+      <c r="F41" s="78"/>
+      <c r="G41" s="78"/>
+      <c r="H41" s="78"/>
+      <c r="I41" s="78"/>
     </row>
     <row r="42" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42"/>
-      <c r="B42"/>
-      <c r="C42"/>
-      <c r="D42"/>
-      <c r="E42"/>
-      <c r="F42"/>
-      <c r="G42"/>
-      <c r="H42"/>
-      <c r="I42"/>
+      <c r="B42" s="78"/>
+      <c r="C42" s="78"/>
+      <c r="D42" s="78"/>
+      <c r="E42" s="78"/>
+      <c r="F42" s="78"/>
+      <c r="G42" s="78"/>
+      <c r="H42" s="78"/>
+      <c r="I42" s="78"/>
     </row>
     <row r="43" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43"/>
-      <c r="B43"/>
-      <c r="C43"/>
-      <c r="D43"/>
-      <c r="E43"/>
-      <c r="F43"/>
-      <c r="G43"/>
-      <c r="H43"/>
-      <c r="I43"/>
+      <c r="B43" s="78"/>
+      <c r="C43" s="78"/>
+      <c r="D43" s="78"/>
+      <c r="E43" s="78"/>
+      <c r="F43" s="78"/>
+      <c r="G43" s="78"/>
+      <c r="H43" s="78"/>
+      <c r="I43" s="78"/>
     </row>
     <row r="44" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44"/>
-      <c r="B44"/>
-      <c r="C44"/>
-      <c r="D44"/>
-      <c r="E44"/>
-      <c r="F44"/>
-      <c r="G44"/>
-      <c r="H44"/>
-      <c r="I44"/>
+      <c r="B44" s="78"/>
+      <c r="C44" s="78"/>
+      <c r="D44" s="78"/>
+      <c r="E44" s="78"/>
+      <c r="F44" s="78"/>
+      <c r="G44" s="78"/>
+      <c r="H44" s="78"/>
+      <c r="I44" s="78"/>
     </row>
     <row r="45" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45"/>
-      <c r="B45"/>
-      <c r="C45"/>
-      <c r="D45"/>
-      <c r="E45"/>
-      <c r="F45"/>
-      <c r="G45"/>
-      <c r="H45"/>
-      <c r="I45"/>
+      <c r="B45" s="78"/>
+      <c r="C45" s="78"/>
+      <c r="D45" s="78"/>
+      <c r="E45" s="78"/>
+      <c r="F45" s="78"/>
+      <c r="G45" s="78"/>
+      <c r="H45" s="78"/>
+      <c r="I45" s="78"/>
     </row>
     <row r="46" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46"/>
-      <c r="B46"/>
-      <c r="C46"/>
-      <c r="D46"/>
-      <c r="E46"/>
-      <c r="F46"/>
-      <c r="G46"/>
-      <c r="H46"/>
-      <c r="I46"/>
+      <c r="B46" s="78"/>
+      <c r="C46" s="78"/>
+      <c r="D46" s="78"/>
+      <c r="E46" s="78"/>
+      <c r="F46" s="78"/>
+      <c r="G46" s="78"/>
+      <c r="H46" s="78"/>
+      <c r="I46" s="78"/>
     </row>
     <row r="47" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47"/>
-      <c r="B47"/>
-      <c r="C47"/>
-      <c r="D47"/>
-      <c r="E47"/>
-      <c r="F47"/>
-      <c r="G47"/>
-      <c r="H47"/>
-      <c r="I47"/>
+      <c r="B47" s="78"/>
+      <c r="C47" s="78"/>
+      <c r="D47" s="78"/>
+      <c r="E47" s="78"/>
+      <c r="F47" s="78"/>
+      <c r="G47" s="78"/>
+      <c r="H47" s="78"/>
+      <c r="I47" s="78"/>
     </row>
     <row r="48" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48"/>
-      <c r="B48"/>
-      <c r="C48"/>
-      <c r="D48"/>
-      <c r="E48"/>
-      <c r="F48"/>
-      <c r="G48"/>
-      <c r="H48"/>
-      <c r="I48"/>
+      <c r="B48" s="78"/>
+      <c r="C48" s="78"/>
+      <c r="D48" s="78"/>
+      <c r="E48" s="78"/>
+      <c r="F48" s="78"/>
+      <c r="G48" s="78"/>
+      <c r="H48" s="78"/>
+      <c r="I48" s="78"/>
     </row>
     <row r="49" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49"/>
-      <c r="B49"/>
-      <c r="C49"/>
-      <c r="D49"/>
-      <c r="E49"/>
-      <c r="F49"/>
-      <c r="G49"/>
-      <c r="H49"/>
-      <c r="I49"/>
+      <c r="B49" s="78"/>
+      <c r="C49" s="78"/>
+      <c r="D49" s="78"/>
+      <c r="E49" s="78"/>
+      <c r="F49" s="78"/>
+      <c r="G49" s="78"/>
+      <c r="H49" s="78"/>
+      <c r="I49" s="78"/>
     </row>
     <row r="50" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50"/>
-      <c r="B50"/>
-      <c r="C50"/>
-      <c r="D50"/>
-      <c r="E50"/>
-      <c r="F50"/>
-      <c r="G50"/>
-      <c r="H50"/>
-      <c r="I50"/>
+      <c r="B50" s="78"/>
+      <c r="C50" s="78"/>
+      <c r="D50" s="78"/>
+      <c r="E50" s="78"/>
+      <c r="F50" s="78"/>
+      <c r="G50" s="78"/>
+      <c r="H50" s="78"/>
+      <c r="I50" s="78"/>
     </row>
   </sheetData>
   <sheetProtection insertRows="0" sort="0" autoFilter="0"/>

</xml_diff>